<commit_message>
PSV: per-case back pressure + inlet/outlet line sizing sheets
Every active scenario now gets its own built-up back-pressure
iteration (Kb, outlet-line dP at that case's own flow/properties)
and inlet-line dP, plus a dedicated CASE_<code> results sheet with
relieving conditions, API 520 sizing detail, orifice selection,
back-pressure and inlet-line (3% rule) checks. SCENARIO_RESULTS
links to each case sheet, and SUMMARY/COMPLIANCE rendering is now
shared via _result_rows with PASS/FAIL coloring.
</commit_message>
<xml_diff>
--- a/PSV/psv_output_PSV-101.xlsx
+++ b/PSV/psv_output_PSV-101.xlsx
@@ -1,16 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SUMMARY" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SCENARIO_RESULTS" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EQUIPMENT_CHECK" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NOTES" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="SUMMARY" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="SCENARIO_RESULTS" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="CASE_BO" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="CASE_FIRE" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="CASE_LOC" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="CASE_BOILUP" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="EQUIPMENT_CHECK" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="NOTES" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -71,6 +75,12 @@
       <name val="Calibri"/>
       <color rgb="00404040"/>
       <sz val="8"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="000563C1"/>
+      <sz val="8"/>
+      <u val="single"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -148,7 +158,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -183,6 +193,9 @@
     <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -198,6 +211,9 @@
     <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -207,7 +223,7 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -586,7 +602,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>PSV SIZING SUMMARY — PSV-101   |   units: FPS   |   11-Jun-2026 18:21</t>
+          <t>PSV SIZING SUMMARY — PSV-101   |   units: FPS   |   12-Jun-2026 02:48</t>
         </is>
       </c>
     </row>
@@ -912,7 +928,8 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="E26" s="5" t="inlineStr">
+      <c r="D26" s="5" t="inlineStr"/>
+      <c r="E26" s="6" t="inlineStr">
         <is>
           <t>set 250.0 vs MAWP 250.0 psia</t>
         </is>
@@ -929,7 +946,8 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="E27" s="5" t="inlineStr">
+      <c r="D27" s="5" t="inlineStr"/>
+      <c r="E27" s="6" t="inlineStr">
         <is>
           <t>Design: 258.8345 psi (g)</t>
         </is>
@@ -946,7 +964,8 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="E28" s="5" t="inlineStr">
+      <c r="D28" s="5" t="inlineStr"/>
+      <c r="E28" s="6" t="inlineStr">
         <is>
           <t>Fire: 284.7179 psi (g)</t>
         </is>
@@ -963,7 +982,8 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="E29" s="5" t="inlineStr">
+      <c r="D29" s="5" t="inlineStr"/>
+      <c r="E29" s="6" t="inlineStr">
         <is>
           <t>Design: 258.8345 psi (g)</t>
         </is>
@@ -980,7 +1000,8 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="E30" s="5" t="inlineStr">
+      <c r="D30" s="5" t="inlineStr"/>
+      <c r="E30" s="6" t="inlineStr">
         <is>
           <t>Design: 258.8345 psi (g)</t>
         </is>
@@ -997,7 +1018,8 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="E31" s="5" t="inlineStr">
+      <c r="D31" s="5" t="inlineStr"/>
+      <c r="E31" s="6" t="inlineStr">
         <is>
           <t>total BP = 0.0% of set</t>
         </is>
@@ -1014,7 +1036,8 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="E32" s="5" t="inlineStr">
+      <c r="D32" s="5" t="inlineStr"/>
+      <c r="E32" s="6" t="inlineStr">
         <is>
           <t>inlet dP = 0.00% of set</t>
         </is>
@@ -1031,7 +1054,8 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="E33" s="5" t="inlineStr">
+      <c r="D33" s="5" t="inlineStr"/>
+      <c r="E33" s="6" t="inlineStr">
         <is>
           <t>min design P = 250.0 psia</t>
         </is>
@@ -1063,7 +1087,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:N16"/>
+  <dimension ref="B1:O16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="2" max="2"/>
@@ -1078,7 +1102,8 @@
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
-    <col width="70" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="70" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -1151,6 +1176,11 @@
       </c>
       <c r="N3" s="9" t="inlineStr">
         <is>
+          <t>Case Sheet</t>
+        </is>
+      </c>
+      <c r="O3" s="9" t="inlineStr">
+        <is>
           <t>Notes</t>
         </is>
       </c>
@@ -1206,6 +1236,11 @@
       </c>
       <c r="N4" s="12" t="inlineStr">
         <is>
+          <t>CASE_BO</t>
+        </is>
+      </c>
+      <c r="O4" s="13" t="inlineStr">
+        <is>
           <t>allowable: 110% set</t>
         </is>
       </c>
@@ -1261,442 +1296,482 @@
       </c>
       <c r="N5" s="12" t="inlineStr">
         <is>
+          <t>CASE_FIRE</t>
+        </is>
+      </c>
+      <c r="O5" s="13" t="inlineStr">
+        <is>
           <t>allowable: 121% set (fire); wetted area (calc) = 33.11 m²; F = 1.000; Q = 761.8 kW; vapor-only screen: dia &lt; 3.0 m and level &lt; 85% expanded volume</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B6" s="14" t="inlineStr">
         <is>
           <t>CV</t>
         </is>
       </c>
-      <c r="C6" s="13" t="inlineStr">
+      <c r="C6" s="14" t="inlineStr">
         <is>
           <t>Control Valve Failure</t>
         </is>
       </c>
-      <c r="D6" s="13" t="inlineStr">
+      <c r="D6" s="14" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="E6" s="13" t="inlineStr">
+      <c r="E6" s="14" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
       </c>
-      <c r="F6" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G6" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H6" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I6" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J6" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K6" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L6" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M6" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N6" s="14" t="inlineStr"/>
+      <c r="F6" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G6" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H6" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I6" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J6" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K6" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L6" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M6" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N6" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O6" s="15" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B7" s="14" t="inlineStr">
         <is>
           <t>GASBB</t>
         </is>
       </c>
-      <c r="C7" s="13" t="inlineStr">
+      <c r="C7" s="14" t="inlineStr">
         <is>
           <t>Gas Blowby / Check-Valve Reverse Flow</t>
         </is>
       </c>
-      <c r="D7" s="13" t="inlineStr">
+      <c r="D7" s="14" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="E7" s="13" t="inlineStr">
+      <c r="E7" s="14" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
       </c>
-      <c r="F7" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G7" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H7" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I7" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J7" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K7" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L7" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M7" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N7" s="14" t="inlineStr"/>
+      <c r="F7" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G7" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H7" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I7" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J7" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K7" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L7" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M7" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N7" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O7" s="15" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="B8" s="13" t="inlineStr">
+      <c r="B8" s="14" t="inlineStr">
         <is>
           <t>THERM</t>
         </is>
       </c>
-      <c r="C8" s="13" t="inlineStr">
+      <c r="C8" s="14" t="inlineStr">
         <is>
           <t>Thermal (Hydraulic) Expansion</t>
         </is>
       </c>
-      <c r="D8" s="13" t="inlineStr">
+      <c r="D8" s="14" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="E8" s="13" t="inlineStr">
+      <c r="E8" s="14" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
       </c>
-      <c r="F8" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G8" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H8" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I8" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J8" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K8" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L8" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M8" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N8" s="14" t="inlineStr"/>
+      <c r="F8" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G8" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H8" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I8" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J8" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K8" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L8" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M8" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N8" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O8" s="15" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="B9" s="13" t="inlineStr">
+      <c r="B9" s="14" t="inlineStr">
         <is>
           <t>TUBE</t>
         </is>
       </c>
-      <c r="C9" s="13" t="inlineStr">
+      <c r="C9" s="14" t="inlineStr">
         <is>
           <t>HX Tube Rupture / Leak</t>
         </is>
       </c>
-      <c r="D9" s="13" t="inlineStr">
+      <c r="D9" s="14" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="E9" s="13" t="inlineStr">
+      <c r="E9" s="14" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
       </c>
-      <c r="F9" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G9" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H9" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I9" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J9" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K9" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L9" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M9" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N9" s="14" t="inlineStr"/>
+      <c r="F9" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G9" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H9" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I9" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J9" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K9" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L9" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M9" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N9" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O9" s="15" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B10" s="14" t="inlineStr">
         <is>
           <t>UTIL</t>
         </is>
       </c>
-      <c r="C10" s="13" t="inlineStr">
+      <c r="C10" s="14" t="inlineStr">
         <is>
           <t>Utility Failure / Loss of Cooling</t>
         </is>
       </c>
-      <c r="D10" s="13" t="inlineStr">
+      <c r="D10" s="14" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="E10" s="13" t="inlineStr">
+      <c r="E10" s="14" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
       </c>
-      <c r="F10" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G10" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H10" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I10" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J10" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K10" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L10" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M10" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N10" s="14" t="inlineStr"/>
+      <c r="F10" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G10" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H10" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I10" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J10" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K10" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L10" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M10" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N10" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O10" s="15" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="B11" s="15" t="inlineStr">
+      <c r="B11" s="16" t="inlineStr">
         <is>
           <t>LOC</t>
         </is>
       </c>
-      <c r="C11" s="15" t="inlineStr">
+      <c r="C11" s="16" t="inlineStr">
         <is>
           <t>Tower Loss of Condensing (HMVRAF)</t>
         </is>
       </c>
-      <c r="D11" s="15" t="inlineStr">
+      <c r="D11" s="16" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="E11" s="15" t="inlineStr">
+      <c r="E11" s="16" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
       </c>
-      <c r="F11" s="16" t="n">
+      <c r="F11" s="17" t="n">
         <v>258.8345</v>
       </c>
-      <c r="G11" s="16" t="n">
+      <c r="G11" s="17" t="n">
         <v>273.5304</v>
       </c>
-      <c r="H11" s="16" t="n">
+      <c r="H11" s="17" t="n">
         <v>268.9</v>
       </c>
-      <c r="I11" s="15" t="inlineStr">
+      <c r="I11" s="16" t="inlineStr">
         <is>
           <t>Two-Phase</t>
         </is>
       </c>
-      <c r="J11" s="16" t="n">
+      <c r="J11" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="K11" s="16" t="n">
+      <c r="K11" s="17" t="n">
         <v>80000</v>
       </c>
-      <c r="L11" s="16" t="n">
+      <c r="L11" s="17" t="n">
         <v>5.6471</v>
       </c>
-      <c r="M11" s="15" t="inlineStr">
+      <c r="M11" s="16" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="N11" s="17" t="inlineStr">
-        <is>
-          <t>allowable: 110% set; props: HMB:HMB.xlsx:T801-OH; HMVRAF flashed adiabatically to relief P: x=0.000; Leung ω = 114.436; Leung ω = 114.436</t>
+      <c r="N11" s="18" t="inlineStr">
+        <is>
+          <t>CASE_LOC</t>
+        </is>
+      </c>
+      <c r="O11" s="19" t="inlineStr">
+        <is>
+          <t>allowable: 110% set; props: HMB:HMB.xlsx:T801-OH; HMVRAF flashed adiabatically to relief P: x=0.000; ⚠ relief P exceeds the HMB stream reference P — verify the linked stream represents relieving conditions; Leung ω = 114.436</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="13" t="inlineStr">
+      <c r="B12" s="14" t="inlineStr">
         <is>
           <t>OVERFILL</t>
         </is>
       </c>
-      <c r="C12" s="13" t="inlineStr">
+      <c r="C12" s="14" t="inlineStr">
         <is>
           <t>Liquid Overfill (Tower §5.6)</t>
         </is>
       </c>
-      <c r="D12" s="13" t="inlineStr">
+      <c r="D12" s="14" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="E12" s="13" t="inlineStr">
+      <c r="E12" s="14" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
       </c>
-      <c r="F12" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G12" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H12" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I12" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J12" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K12" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L12" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M12" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N12" s="14" t="inlineStr"/>
+      <c r="F12" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G12" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H12" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I12" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J12" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K12" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L12" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M12" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N12" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O12" s="15" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="B13" s="10" t="inlineStr">
@@ -1749,208 +1824,2646 @@
       </c>
       <c r="N13" s="12" t="inlineStr">
         <is>
+          <t>CASE_BOILUP</t>
+        </is>
+      </c>
+      <c r="O13" s="13" t="inlineStr">
+        <is>
           <t>allowable: 110% set; props: HMB:HMB.xlsx:T801-OH; no λ available — enter BOILUP λ override</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="13" t="inlineStr">
+      <c r="B14" s="14" t="inlineStr">
         <is>
           <t>ABHEAT</t>
         </is>
       </c>
-      <c r="C14" s="13" t="inlineStr">
+      <c r="C14" s="14" t="inlineStr">
         <is>
           <t>Abnormal Heat Input (§5.4)</t>
         </is>
       </c>
-      <c r="D14" s="13" t="inlineStr">
+      <c r="D14" s="14" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="E14" s="13" t="inlineStr">
+      <c r="E14" s="14" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
       </c>
-      <c r="F14" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G14" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H14" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I14" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J14" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K14" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L14" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M14" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N14" s="14" t="inlineStr"/>
+      <c r="F14" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G14" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H14" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I14" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J14" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K14" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L14" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M14" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N14" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O14" s="15" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="B15" s="13" t="inlineStr">
+      <c r="B15" s="14" t="inlineStr">
         <is>
           <t>RUNAWAY</t>
         </is>
       </c>
-      <c r="C15" s="13" t="inlineStr">
+      <c r="C15" s="14" t="inlineStr">
         <is>
           <t>Runaway Reaction</t>
         </is>
       </c>
-      <c r="D15" s="13" t="inlineStr">
+      <c r="D15" s="14" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="E15" s="13" t="inlineStr">
+      <c r="E15" s="14" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
       </c>
-      <c r="F15" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G15" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H15" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I15" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J15" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K15" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L15" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M15" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N15" s="14" t="inlineStr"/>
+      <c r="F15" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G15" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H15" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I15" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J15" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K15" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L15" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M15" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N15" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O15" s="15" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="B16" s="13" t="inlineStr">
+      <c r="B16" s="14" t="inlineStr">
         <is>
           <t>OTHER</t>
         </is>
       </c>
-      <c r="C16" s="13" t="inlineStr">
+      <c r="C16" s="14" t="inlineStr">
         <is>
           <t>Other / Manual</t>
         </is>
       </c>
-      <c r="D16" s="13" t="inlineStr">
+      <c r="D16" s="14" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="E16" s="13" t="inlineStr">
+      <c r="E16" s="14" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
       </c>
-      <c r="F16" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G16" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H16" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I16" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J16" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K16" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L16" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M16" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N16" s="14" t="inlineStr"/>
+      <c r="F16" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G16" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H16" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I16" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J16" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K16" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L16" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M16" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N16" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O16" s="15" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="B1:N1"/>
+    <mergeCell ref="B1:O1"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N5" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N11" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N13" r:id="rId4"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B1:E42"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="56" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>BO — Blocked Outlet   |   units: FPS</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Relieving Conditions</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="6" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Allowable accumulation pressure (g)</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>258.8345</v>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>psi</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Relieving pressure P1 (abs)</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>273.5304</v>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>psia</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Relieving temperature</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>300</v>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>°F</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Phase</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Vapor</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr"/>
+      <c r="E8" s="6" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Molecular weight</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>g/mol</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Compressibility Z</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="D10" s="5" t="inlineStr"/>
+      <c r="E10" s="6" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>k = Cp/Cv</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="D11" s="5" t="inlineStr"/>
+      <c r="E11" s="6" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Liquid density</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>lb/ft3</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Viscosity</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>cP</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Latent heat</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="n">
+        <v>120</v>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>BTU/lb</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Relief Load</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Relieving mass flow W</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>lb/hr</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Sizing (API 520 Part I)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Molecular weight</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>g/mol</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Compressibility Z</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="D19" s="5" t="inlineStr"/>
+      <c r="E19" s="6" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>k = Cp/Cv</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="D20" s="5" t="inlineStr"/>
+      <c r="E20" s="6" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Mass flux G</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="n">
+        <v>4715.24</v>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>kg/(m²·s)</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Flow regime</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Choked (critical)</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr"/>
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>P2/P1 = 0.054</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Kd (discharge coeff., vapor)</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="n">
+        <v>0.975</v>
+      </c>
+      <c r="D23" s="5" t="inlineStr"/>
+      <c r="E23" s="6" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Kb (back-pressure correction)</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" s="5" t="inlineStr"/>
+      <c r="E24" s="6" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Kc (combination factor)</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" s="5" t="inlineStr"/>
+      <c r="E25" s="6" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Required orifice area</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="n">
+        <v>2.12401</v>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>in2</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Selected orifice (API 526)</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr"/>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t>actual 3.0396 in2</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Back Pressure — Outlet Line (BO flow)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Superimposed back pressure (constant)</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>psi</t>
+        </is>
+      </c>
+      <c r="E29" s="6" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Outlet line dP</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>not evaluated</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr"/>
+      <c r="E30" s="6" t="inlineStr">
+        <is>
+          <t>no line size or no flow — OUTLET_PIPING incomplete</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Built-up back pressure (this case)</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>psi</t>
+        </is>
+      </c>
+      <c r="E31" s="6" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Total back pressure (g)</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>psi</t>
+        </is>
+      </c>
+      <c r="E32" s="6" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Kb (back-pressure correction)</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" s="5" t="inlineStr"/>
+      <c r="E33" s="6" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Total BP vs 10% limit (Conventional)</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr"/>
+      <c r="E34" s="6" t="inlineStr">
+        <is>
+          <t>0.0% of set</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Inlet Line (BO flow) — 3% Rule</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>Inlet line dP</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>not evaluated</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr"/>
+      <c r="E36" s="6" t="inlineStr">
+        <is>
+          <t>no line size or no flow — INLET_PIPING incomplete</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Inlet line pressure drop</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>psi</t>
+        </is>
+      </c>
+      <c r="E37" s="6" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>Inlet dP vs 3% limit</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr"/>
+      <c r="E38" s="6" t="inlineStr">
+        <is>
+          <t>0.00% of set</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Accumulation Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>Allowable within class limit</t>
+        </is>
+      </c>
+      <c r="C40" s="7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr"/>
+      <c r="E40" s="6" t="inlineStr">
+        <is>
+          <t>Design: 258.8345 psi (g)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Notes / Basis</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>allowable: 110% set</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr"/>
+      <c r="D42" s="5" t="inlineStr"/>
+      <c r="E42" s="6" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="B17:E17"/>
+    <mergeCell ref="B41:E41"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="B35:E35"/>
+    <mergeCell ref="B15:E15"/>
+    <mergeCell ref="B39:E39"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="B28:E28"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B1:E45"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="56" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>FIRE — External Fire (API 521)   |   units: FPS</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Relieving Conditions</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Fire</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="6" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Allowable accumulation pressure (g)</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>284.7179</v>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>psi</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Relieving pressure P1 (abs)</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>299.4139</v>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>psia</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Relieving temperature</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>300</v>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>°F</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Phase</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Vapor</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr"/>
+      <c r="E8" s="6" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Molecular weight</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>g/mol</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Compressibility Z</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="D10" s="5" t="inlineStr"/>
+      <c r="E10" s="6" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>k = Cp/Cv</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="D11" s="5" t="inlineStr"/>
+      <c r="E11" s="6" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Liquid density</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>lb/ft3</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Viscosity</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>cP</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Latent heat</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="n">
+        <v>120</v>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>BTU/lb</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Relief Load</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Relieving mass flow W</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="n">
+        <v>21661.34</v>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>lb/hr</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Sizing (API 520 Part I)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Molecular weight</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>g/mol</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Compressibility Z</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="D19" s="5" t="inlineStr"/>
+      <c r="E19" s="6" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>k = Cp/Cv</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="D20" s="5" t="inlineStr"/>
+      <c r="E20" s="6" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Mass flux G</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="n">
+        <v>5161.43</v>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>kg/(m²·s)</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Flow regime</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Choked (critical)</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr"/>
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>P2/P1 = 0.049</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Kd (discharge coeff., vapor)</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="n">
+        <v>0.975</v>
+      </c>
+      <c r="D23" s="5" t="inlineStr"/>
+      <c r="E23" s="6" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Kb (back-pressure correction)</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" s="5" t="inlineStr"/>
+      <c r="E24" s="6" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Kc (combination factor)</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" s="5" t="inlineStr"/>
+      <c r="E25" s="6" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Required orifice area</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="n">
+        <v>0.84063</v>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>in2</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Selected orifice (API 526)</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr"/>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t>actual 1.287 in2</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Back Pressure — Outlet Line (FIRE flow)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Superimposed back pressure (constant)</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>psi</t>
+        </is>
+      </c>
+      <c r="E29" s="6" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Outlet line dP</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>not evaluated</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr"/>
+      <c r="E30" s="6" t="inlineStr">
+        <is>
+          <t>no line size or no flow — OUTLET_PIPING incomplete</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Built-up back pressure (this case)</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>psi</t>
+        </is>
+      </c>
+      <c r="E31" s="6" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Total back pressure (g)</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>psi</t>
+        </is>
+      </c>
+      <c r="E32" s="6" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Kb (back-pressure correction)</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" s="5" t="inlineStr"/>
+      <c r="E33" s="6" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Total BP vs 10% limit (Conventional)</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr"/>
+      <c r="E34" s="6" t="inlineStr">
+        <is>
+          <t>0.0% of set</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Inlet Line (FIRE flow) — 3% Rule</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>Inlet line dP</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>not evaluated</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr"/>
+      <c r="E36" s="6" t="inlineStr">
+        <is>
+          <t>no line size or no flow — INLET_PIPING incomplete</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Inlet line pressure drop</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>psi</t>
+        </is>
+      </c>
+      <c r="E37" s="6" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>Inlet dP vs 3% limit</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr"/>
+      <c r="E38" s="6" t="inlineStr">
+        <is>
+          <t>0.00% of set</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Accumulation Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>Allowable within class limit</t>
+        </is>
+      </c>
+      <c r="C40" s="7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr"/>
+      <c r="E40" s="6" t="inlineStr">
+        <is>
+          <t>Fire: 284.7179 psi (g)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Notes / Basis</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>allowable: 121% set (fire)</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr"/>
+      <c r="D42" s="5" t="inlineStr"/>
+      <c r="E42" s="6" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>wetted area (calc) = 33.11 m²</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr"/>
+      <c r="D43" s="5" t="inlineStr"/>
+      <c r="E43" s="6" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>F = 1.000; Q = 761.8 kW</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr"/>
+      <c r="D44" s="5" t="inlineStr"/>
+      <c r="E44" s="6" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>vapor-only screen: dia &lt; 3.0 m and level &lt; 85% expanded volume</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr"/>
+      <c r="D45" s="5" t="inlineStr"/>
+      <c r="E45" s="6" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="B17:E17"/>
+    <mergeCell ref="B41:E41"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="B35:E35"/>
+    <mergeCell ref="B15:E15"/>
+    <mergeCell ref="B39:E39"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="B28:E28"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B1:E45"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="56" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>LOC — Tower Loss of Condensing (HMVRAF)   ★ GOVERNING CASE   |   units: FPS</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Relieving Conditions</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="6" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Allowable accumulation pressure (g)</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>258.8345</v>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>psi</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Relieving pressure P1 (abs)</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>273.5304</v>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>psia</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Relieving temperature</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>268.9</v>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>°F</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Phase</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Two-Phase</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr"/>
+      <c r="E8" s="6" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Quality x</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="5" t="inlineStr"/>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>mass vapor fraction</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Molecular weight</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>81.36</v>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>g/mol</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Compressibility Z</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>0.901</v>
+      </c>
+      <c r="D11" s="5" t="inlineStr"/>
+      <c r="E11" s="6" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>k = Cp/Cv</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>1.082</v>
+      </c>
+      <c r="D12" s="5" t="inlineStr"/>
+      <c r="E12" s="6" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Vapor density</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>1.0185</v>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>lb/ft3</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Viscosity</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="n">
+        <v>0.0105</v>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>cP</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Relief Load</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Relieving mass flow W</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="n">
+        <v>80000</v>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>lb/hr</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Sizing (API 520 Part I)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Quality x (mass vapor fraction)</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" s="5" t="inlineStr"/>
+      <c r="E18" s="6" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Vapor density (relieving)</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="n">
+        <v>1.0185</v>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>lb/ft3</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Liquid density</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>lb/ft3</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Latent heat</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>BTU/lb</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>not provided — default used</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Leung ω (Annex C)</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="n">
+        <v>114.4361</v>
+      </c>
+      <c r="D22" s="5" t="inlineStr"/>
+      <c r="E22" s="6" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Kd (discharge coeff., two-phase)</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="D23" s="5" t="inlineStr"/>
+      <c r="E23" s="6" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Kc (combination factor)</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" s="5" t="inlineStr"/>
+      <c r="E24" s="6" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Required orifice area</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="n">
+        <v>5.64712</v>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>in2</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Selected orifice (API 526)</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr"/>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>actual 6.3798 in2</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Back Pressure — Outlet Line (LOC flow)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Superimposed back pressure (constant)</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>psi</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Outlet line dP</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>not evaluated</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr"/>
+      <c r="E29" s="6" t="inlineStr">
+        <is>
+          <t>no line size or no flow — OUTLET_PIPING incomplete</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Built-up back pressure (this case)</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>psi</t>
+        </is>
+      </c>
+      <c r="E30" s="6" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Total back pressure (g)</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>psi</t>
+        </is>
+      </c>
+      <c r="E31" s="6" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Kb (back-pressure correction)</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" s="5" t="inlineStr"/>
+      <c r="E32" s="6" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Total BP vs 10% limit (Conventional)</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr"/>
+      <c r="E33" s="6" t="inlineStr">
+        <is>
+          <t>0.0% of set</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Inlet Line (LOC flow) — 3% Rule</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Inlet line dP</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>not evaluated</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr"/>
+      <c r="E35" s="6" t="inlineStr">
+        <is>
+          <t>no line size or no flow — INLET_PIPING incomplete</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>Inlet line pressure drop</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>psi</t>
+        </is>
+      </c>
+      <c r="E36" s="6" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Inlet dP vs 3% limit</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr"/>
+      <c r="E37" s="6" t="inlineStr">
+        <is>
+          <t>0.00% of set</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Accumulation Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>Allowable within class limit</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr"/>
+      <c r="E39" s="6" t="inlineStr">
+        <is>
+          <t>Design: 258.8345 psi (g)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Notes / Basis</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>allowable: 110% set</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr"/>
+      <c r="D41" s="5" t="inlineStr"/>
+      <c r="E41" s="6" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>props: HMB:HMB.xlsx:T801-OH</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr"/>
+      <c r="D42" s="5" t="inlineStr"/>
+      <c r="E42" s="6" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>HMVRAF flashed adiabatically to relief P: x=0.000</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr"/>
+      <c r="D43" s="5" t="inlineStr"/>
+      <c r="E43" s="6" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>⚠ relief P exceeds the HMB stream reference P — verify the linked stream represents relieving conditions</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr"/>
+      <c r="D44" s="5" t="inlineStr"/>
+      <c r="E44" s="6" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>Leung ω = 114.436</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr"/>
+      <c r="D45" s="5" t="inlineStr"/>
+      <c r="E45" s="6" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="B17:E17"/>
+    <mergeCell ref="B27:E27"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="B40:E40"/>
+    <mergeCell ref="B38:E38"/>
+    <mergeCell ref="B15:E15"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="B34:E34"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B1:E43"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="56" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>BOILUP — Liquid Boil-Up (Power Failure §5.7)   |   units: FPS</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Relieving Conditions</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="6" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Allowable accumulation pressure (g)</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>258.8345</v>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>psi</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Relieving pressure P1 (abs)</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>273.5304</v>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>psia</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Relieving temperature</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>343.9</v>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>°F</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Phase</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Vapor</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr"/>
+      <c r="E8" s="6" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Molecular weight</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>75.59</v>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>g/mol</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Compressibility Z</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>0.901</v>
+      </c>
+      <c r="D10" s="5" t="inlineStr"/>
+      <c r="E10" s="6" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>k = Cp/Cv</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>1.082</v>
+      </c>
+      <c r="D11" s="5" t="inlineStr"/>
+      <c r="E11" s="6" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Vapor density</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>1.0185</v>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>lb/ft3</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Viscosity</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>0.0105</v>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>cP</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Relief Load</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Relieving mass flow W</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>lb/hr</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Sizing (API 520 Part I)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Molecular weight</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="n">
+        <v>75.59</v>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>g/mol</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Compressibility Z</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="n">
+        <v>0.901</v>
+      </c>
+      <c r="D18" s="5" t="inlineStr"/>
+      <c r="E18" s="6" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>k = Cp/Cv</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="n">
+        <v>1.082</v>
+      </c>
+      <c r="D19" s="5" t="inlineStr"/>
+      <c r="E19" s="6" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Mass flux G</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="n">
+        <v>5600.14</v>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>kg/(m²·s)</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Flow regime</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Choked (critical)</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr"/>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>P2/P1 = 0.054</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Kd (discharge coeff., vapor)</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="n">
+        <v>0.975</v>
+      </c>
+      <c r="D22" s="5" t="inlineStr"/>
+      <c r="E22" s="6" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Kb (back-pressure correction)</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="5" t="inlineStr"/>
+      <c r="E23" s="6" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Kc (combination factor)</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" s="5" t="inlineStr"/>
+      <c r="E24" s="6" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Required orifice area</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>in2</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Selected orifice (API 526)</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr"/>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>actual 0.0 in2</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Back Pressure — Outlet Line (BOILUP flow)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Superimposed back pressure (constant)</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>psi</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Outlet line dP</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>not evaluated</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr"/>
+      <c r="E29" s="6" t="inlineStr">
+        <is>
+          <t>no line size or no flow — OUTLET_PIPING incomplete</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Built-up back pressure (this case)</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>psi</t>
+        </is>
+      </c>
+      <c r="E30" s="6" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Total back pressure (g)</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>psi</t>
+        </is>
+      </c>
+      <c r="E31" s="6" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Kb (back-pressure correction)</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" s="5" t="inlineStr"/>
+      <c r="E32" s="6" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Total BP vs 10% limit (Conventional)</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr"/>
+      <c r="E33" s="6" t="inlineStr">
+        <is>
+          <t>0.0% of set</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Inlet Line (BOILUP flow) — 3% Rule</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Inlet line dP</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>not evaluated</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr"/>
+      <c r="E35" s="6" t="inlineStr">
+        <is>
+          <t>no line size or no flow — INLET_PIPING incomplete</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>Inlet line pressure drop</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>psi</t>
+        </is>
+      </c>
+      <c r="E36" s="6" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Inlet dP vs 3% limit</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr"/>
+      <c r="E37" s="6" t="inlineStr">
+        <is>
+          <t>0.00% of set</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Accumulation Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>Allowable within class limit</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr"/>
+      <c r="E39" s="6" t="inlineStr">
+        <is>
+          <t>Design: 258.8345 psi (g)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Notes / Basis</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>allowable: 110% set</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr"/>
+      <c r="D41" s="5" t="inlineStr"/>
+      <c r="E41" s="6" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>props: HMB:HMB.xlsx:T801-OH</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr"/>
+      <c r="D42" s="5" t="inlineStr"/>
+      <c r="E42" s="6" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>no λ available — enter BOILUP λ override</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr"/>
+      <c r="D43" s="5" t="inlineStr"/>
+      <c r="E43" s="6" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="B40:E40"/>
+    <mergeCell ref="B27:E27"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="B38:E38"/>
+    <mergeCell ref="B16:E16"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="B34:E34"/>
+    <mergeCell ref="B14:E14"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1976,68 +4489,68 @@
       </c>
     </row>
     <row r="3">
-      <c r="B3" s="18" t="inlineStr">
+      <c r="B3" s="20" t="inlineStr">
         <is>
           <t>Tag</t>
         </is>
       </c>
-      <c r="C3" s="18" t="inlineStr">
+      <c r="C3" s="20" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="D3" s="18" t="inlineStr">
+      <c r="D3" s="20" t="inlineStr">
         <is>
           <t>Design P (psia)</t>
         </is>
       </c>
-      <c r="E3" s="18" t="inlineStr">
+      <c r="E3" s="20" t="inlineStr">
         <is>
           <t>MAWP (psia)</t>
         </is>
       </c>
-      <c r="F3" s="18" t="inlineStr">
+      <c r="F3" s="20" t="inlineStr">
         <is>
           <t>EL (ft)</t>
         </is>
       </c>
-      <c r="G3" s="18" t="inlineStr">
+      <c r="G3" s="20" t="inlineStr">
         <is>
           <t>Design P ≥ Set P?</t>
         </is>
       </c>
-      <c r="H3" s="18" t="inlineStr">
+      <c r="H3" s="20" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="19" t="inlineStr">
+      <c r="B4" s="21" t="inlineStr">
         <is>
           <t>V-101</t>
         </is>
       </c>
-      <c r="C4" s="19" t="inlineStr">
+      <c r="C4" s="21" t="inlineStr">
         <is>
           <t>Vertical Vessel</t>
         </is>
       </c>
-      <c r="D4" s="19" t="n">
+      <c r="D4" s="21" t="n">
         <v>250</v>
       </c>
-      <c r="E4" s="19" t="n">
+      <c r="E4" s="21" t="n">
         <v>250</v>
       </c>
-      <c r="F4" s="19" t="n">
+      <c r="F4" s="21" t="n">
         <v>10</v>
       </c>
-      <c r="G4" s="19" t="inlineStr">
+      <c r="G4" s="21" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="H4" s="19" t="inlineStr">
+      <c r="H4" s="21" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2051,180 +4564,208 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:A26"/>
+  <dimension ref="A2:A30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="2">
-      <c r="A2" s="20" t="inlineStr">
+      <c r="A2" s="22" t="inlineStr">
         <is>
           <t>METHODOLOGY &amp; ASSUMPTIONS</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="21" t="inlineStr"/>
+      <c r="A3" s="23" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="21" t="inlineStr">
+      <c r="A4" s="23" t="inlineStr">
         <is>
           <t>· Sizing per API 520 Part I: vapor (isentropic nozzle, critical/subcritical),</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="21" t="inlineStr">
+      <c r="A5" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">  liquid (theoretical orifice with Kd/Kw/Kc/Kv), two-phase (Leung omega, Annex C).</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="21" t="inlineStr">
+      <c r="A6" s="23" t="inlineStr">
         <is>
           <t>· Fire per API 521 §5.15 with project convention Q = F·43200·A^0.82 [W, m²];</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="21" t="inlineStr">
+      <c r="A7" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">  vapor-only screening and the two-phase swell estimate per methodology §3.10.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="21" t="inlineStr">
+      <c r="A8" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">  The two-phase W₂ uses a homogeneous-vessel swell approximation — review</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="21" t="inlineStr">
+      <c r="A9" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">  against the corporate energy/swell balance before final design.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="21" t="inlineStr">
+      <c r="A10" s="23" t="inlineStr">
         <is>
           <t>· Contingency classes per §2: Design 110%/116%, Fire 121%, Remote =</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="21" t="inlineStr">
+      <c r="A11" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">  min(HTF×DP, corrected test pressure) with 1.3×MAWP fallback.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="21" t="inlineStr">
+      <c r="A12" s="23" t="inlineStr">
         <is>
           <t>· CV failure per §3.3: design = bypass at 50% of normal operating Cv;</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="21" t="inlineStr">
+      <c r="A13" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">  remote = bypass 100% open at rated Cv.  ISA/IEC 60534 flow equations.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="21" t="inlineStr">
+      <c r="A14" s="23" t="inlineStr">
         <is>
           <t>· Check-valve reverse flow per §3.7 (6% / 2% of minimum internal diameter).</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="21" t="inlineStr">
+      <c r="A15" s="23" t="inlineStr">
         <is>
           <t>· Tower methods per §5: LOC = HMVRAF flashed adiabatically; boil-up =</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="21" t="inlineStr">
+      <c r="A16" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">  two-flash λ; overfill quality = max reboiler + max feed vapor; abnormal</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="21" t="inlineStr">
+      <c r="A17" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">  heat = duty-ratio scaling with optional LMTD pinch credit (§5.1).</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="21" t="inlineStr">
+      <c r="A18" s="23" t="inlineStr">
         <is>
           <t>· Static-elevation corrected set pressure per 'PSV Inputs plus'.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="21" t="inlineStr">
+      <c r="A19" s="23" t="inlineStr">
         <is>
           <t>· Relieving temperature uses bubble/dew/adiabatic-flash of the linked HMB</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="21" t="inlineStr">
+      <c r="A20" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">  composition (hydraulics flash engine) where available.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="21" t="inlineStr">
+      <c r="A21" s="23" t="inlineStr">
         <is>
           <t>· INLET/OUTLET piping use a single-line Darcy model — for relief circuits</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="21" t="inlineStr">
+      <c r="A22" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">  run the hydraulics engine and paste the dP into the override cells.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="21" t="inlineStr"/>
+      <c r="A23" s="23" t="inlineStr">
+        <is>
+          <t>· Every active scenario gets its own CASE_&lt;code&gt; sheet with a full</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="21" t="inlineStr">
+      <c r="A24" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  back-pressure iteration (Kb, built-up BP, outlet-line v/Re/f at that</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  case's relief rate/properties) and inlet-line dP through the shared</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  INLET/OUTLET piping geometry — see SCENARIO_RESULTS 'Case Sheet' links.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="23" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="23" t="inlineStr">
         <is>
           <t>VERIFY all results against API 520/521 and the corporate practice before</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="21" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="23" t="inlineStr">
         <is>
           <t>issuing for design.  This workbook is a calculation aid, not a substitute</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="21" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="23" t="inlineStr">
         <is>
           <t>for engineering review.</t>
         </is>

</xml_diff>